<commit_message>
HKUST: minimum 4 courses (12 credits); BA moved to to-check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_3_NotInReviewEntry_OK.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_3_NotInReviewEntry_OK.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Rows removed (not usable)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Geography BA'!$A$1:$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Geography BA'!$A$1:$K$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Geography BSc'!$A$1:$K$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rows removed (not usable)'!$A$1:$K$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rows removed (not usable)'!$A$1:$K$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -72,12 +72,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00D9F2D0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9F2D0"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -568,21 +568,21 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Meets minimum, little choice: 3 modules with confirmed 2026/27 term, 3 needed (+6 more with unverified term)</t>
+          <t>OK: 6 modules with confirmed 2026/27 term, 4 needed (+2 more with unverified term)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -591,83 +591,46 @@
         </is>
       </c>
       <c r="H5" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology</t>
+          <t>Washington State University</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>OK: 6 modules with confirmed 2026/27 term, 3 needed (+2 more with unverified term)</t>
+        <v>4</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Meets minimum, little choice: 4 modules with confirmed Fall 2026 term, 4 needed. WSU has no Geography department - modules are from School of the Environment / Sociology; department to confirm content fit.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Semester 1 or 2 </t>
+          <t>Fall Semester [Sep-Dec)</t>
         </is>
       </c>
       <c r="H6" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Washington State University</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Meets minimum, little choice: 4 modules with confirmed Fall 2026 term, 4 needed. WSU has no Geography department - modules are from School of the Environment / Sociology; department to confirm content fit.</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Fall Semester [Sep-Dec)</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="I7" s="3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -682,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -758,7 +721,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
+          <t>Washington State University — USA</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -768,7 +731,7 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
+          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -778,12 +741,12 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>ENVR2020 Urban Air Pollution (3 credits)</t>
+          <t>SOC 338 Environmental Inequality and Justice (3 credits)</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -793,131 +756,131 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Fall 2026 - HKUST takes students in either semester</t>
+          <t>Fall 2026 (Pullman) - verified in WSU Schedule of Classes Oct 2026</t>
         </is>
       </c>
       <c r="I2" s="6" t="n"/>
       <c r="J2" s="6" t="inlineStr">
         <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/ENVR | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM VERIFIED Oct 2026: Fall 2026 - HKUST takes students in either semester [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
+          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Washington State University — USA</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>SOC310 Development of Social Theory</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Fall 2026 (Aug 24 - Dec 11, Pullman)</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="n"/>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/SOC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM VERIFIED Oct 2026: Fall 2026 (Aug 24 - Dec 11, Pullman) [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Washington State University — USA</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Geography BA</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>ENVR2060 From Trash to Treasure: Transforming Waste into Resources (3 credits)</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>SOE 312 Natural Resources, Society, and the Environment (3 credits)</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>2026-27 catalogue (term set at registration)</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/ENVR | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Not in Fall 2026 schedule; Spring 2027 schedule not yet published (HKUST takes either semester) [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>ENVR3005 Environmental Risks: Principles and Practices (3 credits)</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>2026-27 catalogue (term set at registration)</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/ENVR | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Not in Fall 2026 schedule; Spring 2027 schedule not yet published (HKUST takes either semester) [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Fall 2026 (Pullman) - verified in WSU Schedule of Classes Oct 2026</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Host: https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
+          <t>Washington State University — USA</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -937,12 +900,12 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>ENVR3410 Economics for Environmental Policy and Management (3 credits)</t>
+          <t>SOE 487 Human Dimensions of Natural Resources (3 credits)</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 4</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -952,500 +915,23 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Fall 2026 - HKUST takes students in either semester</t>
+          <t>Fall 2026 (Pullman) - verified in WSU Schedule of Classes Oct 2026</t>
         </is>
       </c>
       <c r="I5" s="6" t="n"/>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/ENVR | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM VERIFIED Oct 2026: Fall 2026 - HKUST takes students in either semester [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>SOSC2299 The Rise and Fall of Globalization (3 credits)</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>2026-27 catalogue (term set at registration)</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/SOSC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Not in Fall 2026 schedule; Spring 2027 schedule not yet published (HKUST takes either semester) [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>SOSC2330 Environmental Politics and Policy (3 credits)</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>2026-27 catalogue (term set at registration)</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="n"/>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/SOSC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Not in Fall 2026 schedule; Spring 2027 schedule not yet published (HKUST takes either semester) [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>SOSC2740 Gender and Society (3 credits)</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Fall 2026 - HKUST takes students in either semester</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/SOSC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM VERIFIED Oct 2026: Fall 2026 - HKUST takes students in either semester [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>SOSC3250 Gender and Development (3 credits)</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>2026-27 catalogue (term set at registration)</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="n"/>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/SOSC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Not in Fall 2026 schedule; Spring 2027 schedule not yet published (HKUST takes either semester) [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>SOSC3880 Social Inequality and Social Mobility (3 credits)</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>2026-27 catalogue (term set at registration)</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="n"/>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/SOSC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Not in Fall 2026 schedule; Spring 2027 schedule not yet published (HKUST takes either semester) [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Washington State University — USA</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>SOC 338 Environmental Inequality and Justice (3 credits)</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>Fall 2026 (Pullman) - verified in WSU Schedule of Classes Oct 2026</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>Host: https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
           <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Washington State University — USA</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>SOC310 Development of Social Theory</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>Fall 2026 (Aug 24 - Dec 11, Pullman)</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/SOC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM VERIFIED Oct 2026: Fall 2026 (Aug 24 - Dec 11, Pullman) [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Washington State University — USA</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>SOE 312 Natural Resources, Society, and the Environment (3 credits)</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>Fall 2026 (Pullman) - verified in WSU Schedule of Classes Oct 2026</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>Host: https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="inlineStr">
-        <is>
-          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Washington State University — USA</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>SOE 487 Human Dimensions of Natural Resources (3 credits)</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Level 4</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>Fall 2026 (Pullman) - verified in WSU Schedule of Classes Oct 2026</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>Host: https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K14" s="7" t="inlineStr">
-        <is>
-          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K14"/>
+  <autoFilter ref="A1:K5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1530,159 +1016,159 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>CIVL4660 Geospatial Science and Technology for Smart City (3 credits)</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Level 4</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Fall 2026 - verified in HKUST class schedule Oct 2026 (HKUST takes students in either semester)</t>
         </is>
       </c>
-      <c r="I2" s="7" t="n"/>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>Host: https://w5.ab.ust.hk/wcq/cgi-bin/2610/ (HKUST Class Schedule, Fall 2026-27) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>ENVR2010 Environmental Science Fundamentals (3 credits)</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Level 2</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Fall 2026 - verified in HKUST class schedule Oct 2026 (HKUST takes students in either semester)</t>
         </is>
       </c>
-      <c r="I3" s="7" t="n"/>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>Host: https://w5.ab.ust.hk/wcq/cgi-bin/2610/ (HKUST Class Schedule, Fall 2026-27) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>ENVR2020 Urban Air Pollution (3 credits)</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Level 2</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Fall 2026 - HKUST takes students in either semester</t>
         </is>
       </c>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/ENVR | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM VERIFIED Oct 2026: Fall 2026 - HKUST takes students in either semester [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
         </is>
@@ -1795,159 +1281,159 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>ENVR3010S Nature-based Solutions (3 credits)</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Fall 2026 - verified in HKUST class schedule Oct 2026 (HKUST takes students in either semester)</t>
         </is>
       </c>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>Host: https://w5.ab.ust.hk/wcq/cgi-bin/2610/ (HKUST Class Schedule, Fall 2026-27) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>ENVR3220 Energy Sources and Usage (3 credits)</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Fall 2026 - HKUST takes students in either semester</t>
         </is>
       </c>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/ENVR | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM VERIFIED Oct 2026: Fall 2026 - HKUST takes students in either semester [https://w5.ab.ust.hk/wcq/cgi-bin/2610/]</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>OCES2003 Descriptive Physical Oceanography (3 credits)</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Level 2</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Fall 2026 - verified in HKUST class schedule Oct 2026 (HKUST takes students in either semester)</t>
         </is>
       </c>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Host: https://w5.ab.ust.hk/wcq/cgi-bin/2610/ (HKUST Class Schedule, Fall 2026-27) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
         </is>
@@ -1965,7 +1451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2041,7 +1527,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology — Hong Kong (SAR)</t>
+          <t>Washington State University — USA</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -2051,7 +1537,7 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
+          <t>SOES220 CITIES AND REGIONS</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
@@ -2061,12 +1547,12 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>SOSC3130 Hong Kong Culture (3 credits)</t>
+          <t>ASIA220 Global Issues, Regional Realities</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
@@ -2076,18 +1562,18 @@
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Fall 2026 - HKUST takes students in either semester</t>
+          <t>Term not stated in catalogue</t>
         </is>
       </c>
       <c r="I2" s="8" t="n"/>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>Host: https://prog-crs.hkust.edu.hk/ugcourse/2026-27/SOSC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/ASI | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT USABLE (language of tuition): Taught in Cantonese — Medium of instruction: Cantonese; requires Chinese reading - not usable [https://w5.ab.ust.hk/wcq/cgi-bin/2610/subject/SOSC]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
         </is>
       </c>
     </row>
@@ -2104,7 +1590,7 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>SOES220 CITIES AND REGIONS</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -2114,12 +1600,12 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>ASIA220 Global Issues, Regional Realities</t>
+          <t>SOC331 Population, Resources, and the Future</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -2135,7 +1621,7 @@
       <c r="I3" s="8" t="n"/>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/ASI | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/SOC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K3" s="8" t="inlineStr">
@@ -2144,61 +1630,8 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Washington State University — USA</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>SOC331 Population, Resources, and the Future</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>Term not stated in catalogue</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/SOC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
-        </is>
-      </c>
-      <c r="K4" s="8" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:K3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>